<commit_message>
Mark all fixtures as synthetic, ahead of a public push
fixtures/ contains invented vendor policies and a fake questionnaire
with no real-world provenance. Before this repo is pushed publicly,
every fixture file needs to say so plainly so it can't be mistaken for
a real organization's documents by anyone who finds it out of context.
Added a visible notice to the top of the markdown evidence file, a body
paragraph plus generator-script docstring note for the DOCX evidence
file, and workbook properties + an A1 cell comment for the xlsx
questionnaire (chosen over inserting a banner row so the existing row
numbers - already exercised throughout manual testing - don't shift).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/questionnaire_sample.xlsx
+++ b/fixtures/questionnaire_sample.xlsx
@@ -128,6 +128,21 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Questionnaire Responder</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>SYNTHETIC TEST FIXTURE — NOT A REAL QUESTIONNAIRE. Invented for this project's tests; does not represent any real company's questionnaire or vendor.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -515,5 +530,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>